<commit_message>
Seed parked jobs into the joinery drive
Same treatment as the foyle drive: nine jobs stop mid-flow, two with no
fitter's name, six held by one fitter against a load limit of four. The
action queue is now non-empty for all three SMEs, which is the product-level
half of the generalisability claim.
</commit_message>
<xml_diff>
--- a/data/synthetic/messy_joinery/jobs 2026.xlsx
+++ b/data/synthetic/messy_joinery/jobs 2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>15/01/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>18/01/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>19/01/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>22/01/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>26/01/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>25/01/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>27/01/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>28/01/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>30/01/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11/02/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>15/02/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17/02/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>07/02/2026</t>
+          <t>25/03/2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>27/03/2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10/02/2026</t>
+          <t>28/03/2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>13/02/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>22/02/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>19/02/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>22/02/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>27/02/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>06/03/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>20/03/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>22/03/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>21/03/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>18/05/2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>26/05/2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>26/03/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>26/05/2026</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>07/06/2026</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>14/06/2026</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>04/06/2026</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2477,6 +2477,865 @@
       <c r="E76" t="inlineStr">
         <is>
           <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>J-1036</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>QUOTE SENT</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>J-1037</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>QUOTE SENT</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>client to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>J-1038</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>quote sent</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>29/05/2026</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>J-1038</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Quote Accepted</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>02/06/2026</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>supplier late</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>J-1039</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>QUOTE SENT</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>J-1039</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>QUOTE ACCEPTED</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>J-1039</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>site survey</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>J-1039</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MATERIALS ORDERED</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>02/06/2026</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>waiting on glass</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>J-1040</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Quote Sent</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>J-1040</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>quote accepted</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>J-1040</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>site survey</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>J-1040</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Materials Ordered</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>waiting on glass</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>J-1041</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Quote Sent</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>17/05/2026</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>J-1041</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>quote accepted</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>J-1041</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>site survey</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>J-1041</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>materials ordered</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>J-1041</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Site Work Started</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>J-1042</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Quote Sent</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Ciara McCrossan</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>J-1042</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>QUOTE ACCEPTED</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>29/05/2026</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Ciara McCrossan</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>J-1042</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Site Survey</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Ciara McCrossan</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>J-1042</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Materials Ordered </t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>02/06/2026</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Ciara McCrossan</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>J-1042</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Site Work Started </t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Ciara McCrossan</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>J-1042</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>SNAGGING</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Ciara McCrossan</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>supplier late</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>J-1043</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>QUOTE SENT</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>J-1043</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>quote accepted</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done </t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>J-1043</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>SITE SURVEY</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>07/06/2026</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>J-1043</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>materials ordered</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>J-1043</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Site Work Started </t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>J-1043</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SNAGGING</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>J-1043</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>INVOICE SENT</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>J-1044</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Quote Sent</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>J-1044</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>quote accepted</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>sorted</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>J-1044</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Site Survey </t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>02/06/2026</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Mark Deehan</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>tbc</t>
         </is>
       </c>
     </row>

</xml_diff>